<commit_message>
feat(shefish): split PI Number and PO Number on updated templates
SHEFISH PI now writes PI# from PO RECORD and the customer PO# separately, and blocks when PI# is missing.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/customer_profiles/shefish/templates/emax/pi.xlsx
+++ b/customer_profiles/shefish/templates/emax/pi.xlsx
@@ -9,7 +9,7 @@
     <sheet name="PI format" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'PI format'!$A$1:$G$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'PI format'!$A$1:$G$29</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +25,7 @@
     <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="169" formatCode="dd/mmm/yy"/>
   </numFmts>
-  <fonts count="55">
+  <fonts count="52">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -78,16 +78,11 @@
     <font>
       <name val="Arial"/>
       <charset val="134"/>
+      <color rgb="FFFF0000"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <color theme="1"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
+      <name val="宋体"/>
       <charset val="134"/>
       <color rgb="FFFF0000"/>
       <sz val="9"/>
@@ -381,18 +376,6 @@
       <name val="Arial"/>
       <charset val="134"/>
       <color rgb="FF00B0F0"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <color rgb="FFFF0000"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <color rgb="FFFF0000"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -974,319 +957,319 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="11" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="11" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="43" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="9" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="10" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="9" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="6" borderId="11" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="12" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="13" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="7" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="9" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="11" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="12" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="13" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="15" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="19" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="23" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="27" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="31" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="33" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="34" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="35" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="36" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="37" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="38" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="36" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="10" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="11" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="12" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="13" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="34" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="35" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="36" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="37" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="38" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="36" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="33" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="34" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="31" fillId="38" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="35" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="39" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="40" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="38" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="36" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="38" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="41" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="42" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="40" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="38" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="35" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="34" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="30" fillId="38" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="35" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="39" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="40" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="38" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="36" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="38" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="41" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="42" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="40" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="38" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="35" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="35" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="36" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="37" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="36" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="34" fillId="36" borderId="14" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="38" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="39" fillId="0" borderId="15" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="40" fillId="0" borderId="16" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="41" fillId="0" borderId="17" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="41" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="33" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="164" fontId="35" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="33" fillId="36" borderId="14" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="37" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="38" fillId="0" borderId="15" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="39" fillId="0" borderId="16" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="40" fillId="0" borderId="17" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="40" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="36" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="35" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="42" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="36" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="35" fillId="43" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="41" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="42" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="44" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="45" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="46" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="43" fillId="0" borderId="18" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="44" fillId="47" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="45" fillId="48" borderId="19" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="46" fillId="49" borderId="20" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="47" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="47" fillId="0" borderId="21" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="48" fillId="48" borderId="22" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="49" fillId="39" borderId="19" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="50" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="36" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="51" fillId="39" borderId="0" applyAlignment="1">
+    <xf numFmtId="164" fontId="41" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="35" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="34" fillId="43" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="41" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="42" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="44" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="45" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="46" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="42" fillId="0" borderId="18" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="43" fillId="47" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="44" fillId="48" borderId="19" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="45" fillId="49" borderId="20" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="46" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="46" fillId="0" borderId="21" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="47" fillId="48" borderId="22" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="48" fillId="39" borderId="19" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="49" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="35" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="50" fillId="39" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="143">
+  <cellXfs count="137">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1345,17 +1328,27 @@
     <xf numFmtId="165" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="55">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="166" fontId="2" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="55">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="55">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="55">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1366,10 +1359,10 @@
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="76">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="55">
@@ -1379,10 +1372,10 @@
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="88">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="86">
@@ -1448,19 +1441,19 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1472,10 +1465,10 @@
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="57">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="57">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="57">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="57">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="57">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="98">
@@ -1553,16 +1546,26 @@
     <xf numFmtId="165" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="166" fontId="2" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="55">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="55">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1573,10 +1576,10 @@
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="76">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="55">
@@ -1648,17 +1651,8 @@
     <xf numFmtId="165" fontId="1" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="86">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="169" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1669,10 +1663,10 @@
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="57">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="57">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="57">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="57">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="57">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="98">
@@ -1705,33 +1699,6 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="86">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="55">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="55">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="116">
@@ -2159,428 +2126,442 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="11.6"/>
   <cols>
-    <col width="17.75" customWidth="1" style="73" min="1" max="1"/>
-    <col width="16.25" customWidth="1" style="73" min="2" max="2"/>
-    <col width="13.3166666666667" customWidth="1" style="73" min="3" max="3"/>
-    <col width="35.8833333333333" customWidth="1" style="73" min="4" max="4"/>
-    <col width="13.575" customWidth="1" style="73" min="5" max="5"/>
-    <col width="13.125" customWidth="1" style="73" min="6" max="6"/>
-    <col width="16.5" customWidth="1" style="73" min="7" max="7"/>
-    <col width="11.375" customWidth="1" style="74" min="8" max="8"/>
-    <col width="9" customWidth="1" style="73" min="9" max="16384"/>
+    <col width="17.75" customWidth="1" style="76" min="1" max="1"/>
+    <col width="16.25" customWidth="1" style="76" min="2" max="2"/>
+    <col width="13.3166666666667" customWidth="1" style="76" min="3" max="3"/>
+    <col width="35.8833333333333" customWidth="1" style="76" min="4" max="4"/>
+    <col width="13.575" customWidth="1" style="76" min="5" max="5"/>
+    <col width="13.125" customWidth="1" style="76" min="6" max="6"/>
+    <col width="16.5" customWidth="1" style="76" min="7" max="7"/>
+    <col width="11.375" customWidth="1" style="77" min="8" max="8"/>
+    <col width="9" customWidth="1" style="76" min="9" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customFormat="1" customHeight="1" s="75">
-      <c r="A1" s="76" t="inlineStr">
+    <row r="1" ht="25.5" customFormat="1" customHeight="1" s="78">
+      <c r="A1" s="79" t="inlineStr">
         <is>
           <t>E MAX SPORT PTE. LTD.</t>
         </is>
       </c>
-      <c r="H1" s="77" t="n"/>
-    </row>
-    <row r="2" ht="21.95" customFormat="1" customHeight="1" s="75">
-      <c r="A2" s="78" t="inlineStr">
+      <c r="H1" s="80" t="n"/>
+    </row>
+    <row r="2" ht="21.95" customFormat="1" customHeight="1" s="78">
+      <c r="A2" s="81" t="inlineStr">
         <is>
           <t>8 KAKI BUKIT AVENUE 4, #08-32,PREMIER @ KAKI BUKIT, SINGAPORE 415875</t>
         </is>
       </c>
-      <c r="H2" s="77" t="n"/>
-    </row>
-    <row r="3" ht="18.95" customFormat="1" customHeight="1" s="75">
-      <c r="H3" s="77" t="n"/>
-    </row>
-    <row r="4" ht="27.95" customFormat="1" customHeight="1" s="75">
-      <c r="A4" s="79" t="inlineStr">
+      <c r="H2" s="80" t="n"/>
+    </row>
+    <row r="3" ht="18.95" customFormat="1" customHeight="1" s="78">
+      <c r="H3" s="80" t="n"/>
+    </row>
+    <row r="4" ht="27.95" customFormat="1" customHeight="1" s="78">
+      <c r="A4" s="82" t="inlineStr">
         <is>
           <t>PROFORMA INVOICE</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15.95" customFormat="1" customHeight="1" s="75">
-      <c r="A5" s="80" t="n"/>
+    <row r="5" ht="15.95" customFormat="1" customHeight="1" s="78">
+      <c r="A5" s="83" t="n"/>
       <c r="B5" s="13" t="n"/>
-      <c r="D5" s="81" t="n"/>
-      <c r="E5" s="82" t="n"/>
+      <c r="D5" s="84" t="n"/>
+      <c r="E5" s="85" t="n"/>
       <c r="F5" s="16" t="n"/>
       <c r="G5" s="16" t="n"/>
-      <c r="H5" s="83" t="n"/>
-    </row>
-    <row r="6" ht="17" customFormat="1" customHeight="1" s="84">
-      <c r="A6" s="80" t="inlineStr">
+      <c r="H5" s="86" t="n"/>
+    </row>
+    <row r="6" ht="15.95" customFormat="1" customHeight="1" s="78">
+      <c r="A6" s="83" t="n"/>
+      <c r="B6" s="13" t="n"/>
+      <c r="D6" s="84" t="n"/>
+      <c r="E6" s="85" t="n"/>
+      <c r="F6" s="85" t="inlineStr">
+        <is>
+          <t>PI Number:</t>
+        </is>
+      </c>
+      <c r="G6" s="87" t="n"/>
+      <c r="H6" s="88" t="n"/>
+    </row>
+    <row r="7" ht="15.95" customFormat="1" customHeight="1" s="89">
+      <c r="A7" s="83" t="inlineStr">
         <is>
           <t>Incoterm:</t>
         </is>
       </c>
-      <c r="B6" s="137" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>DDP USA</t>
         </is>
       </c>
-      <c r="F6" s="82" t="inlineStr">
-        <is>
-          <t>PI Number:</t>
-        </is>
-      </c>
-      <c r="G6" s="86" t="n"/>
-      <c r="H6" s="102" t="n"/>
-      <c r="I6" s="87" t="n"/>
-    </row>
-    <row r="7" ht="17" customFormat="1" customHeight="1" s="84">
-      <c r="A7" s="80" t="inlineStr">
+      <c r="C7" s="88" t="n"/>
+      <c r="D7" s="83" t="n"/>
+      <c r="F7" s="90" t="inlineStr">
+        <is>
+          <t>PO Number:</t>
+        </is>
+      </c>
+      <c r="G7" s="91" t="n"/>
+      <c r="H7" s="92" t="n"/>
+      <c r="I7" s="93" t="n"/>
+    </row>
+    <row r="8" ht="15.95" customFormat="1" customHeight="1" s="89">
+      <c r="A8" s="83" t="inlineStr">
         <is>
           <t>Payment Terms:</t>
         </is>
       </c>
-      <c r="B7" s="137" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>Net 60 days</t>
         </is>
       </c>
-      <c r="F7" s="82" t="inlineStr">
+      <c r="C8" s="88" t="n"/>
+      <c r="D8" s="83" t="n"/>
+      <c r="F8" s="85" t="inlineStr">
         <is>
           <t>Document Date:</t>
         </is>
       </c>
-      <c r="G7" s="88" t="n"/>
-      <c r="H7" s="107" t="n"/>
-      <c r="I7" s="87" t="n"/>
-    </row>
-    <row r="8" ht="15.95" customFormat="1" customHeight="1" s="84">
-      <c r="D8" s="80" t="n"/>
-      <c r="F8" s="82" t="n"/>
-      <c r="G8" s="82" t="n"/>
-      <c r="H8" s="85" t="n"/>
-      <c r="I8" s="87" t="n"/>
-    </row>
-    <row r="9" ht="17" customFormat="1" customHeight="1" s="84">
-      <c r="A9" s="89" t="inlineStr">
+      <c r="G8" s="94" t="n"/>
+      <c r="H8" s="88" t="n"/>
+      <c r="I8" s="93" t="n"/>
+    </row>
+    <row r="9" ht="15.95" customFormat="1" customHeight="1" s="89">
+      <c r="D9" s="83" t="n"/>
+      <c r="F9" s="85" t="n"/>
+      <c r="G9" s="85" t="n"/>
+      <c r="H9" s="88" t="n"/>
+      <c r="I9" s="93" t="n"/>
+    </row>
+    <row r="10" ht="15.95" customFormat="1" customHeight="1" s="89">
+      <c r="A10" s="95" t="inlineStr">
         <is>
           <t>Bill To:</t>
         </is>
       </c>
-      <c r="B9" s="90" t="inlineStr">
+      <c r="B10" s="96" t="inlineStr">
         <is>
           <t xml:space="preserve">She Fish </t>
         </is>
       </c>
-      <c r="C9" s="135" t="n"/>
-      <c r="D9" s="135" t="n"/>
-      <c r="F9" s="92" t="inlineStr">
+      <c r="C10" s="97" t="n"/>
+      <c r="D10" s="88" t="n"/>
+      <c r="F10" s="98" t="inlineStr">
         <is>
           <t>Ship to:</t>
         </is>
       </c>
-      <c r="G9" s="90" t="inlineStr">
+      <c r="G10" s="96" t="inlineStr">
         <is>
           <t xml:space="preserve">She Fish </t>
         </is>
       </c>
-      <c r="H9" s="135" t="n"/>
-      <c r="I9" s="85" t="n"/>
-    </row>
-    <row r="10" ht="17" customFormat="1" customHeight="1" s="84">
-      <c r="A10" s="93" t="n"/>
-      <c r="B10" s="29" t="inlineStr">
+      <c r="H10" s="97" t="n"/>
+      <c r="I10" s="88" t="n"/>
+    </row>
+    <row r="11" ht="17" customFormat="1" customHeight="1" s="89">
+      <c r="A11" s="99" t="n"/>
+      <c r="B11" s="31" t="inlineStr">
         <is>
           <t>The Fishing Brands, LLC</t>
         </is>
       </c>
-      <c r="C10" s="95" t="n"/>
-      <c r="D10" s="95" t="n"/>
-      <c r="F10" s="82" t="n"/>
-      <c r="G10" s="29" t="inlineStr">
+      <c r="C11" s="31" t="n"/>
+      <c r="D11" s="88" t="n"/>
+      <c r="F11" s="85" t="n"/>
+      <c r="G11" s="31" t="inlineStr">
         <is>
           <t>The Fishing Brands, LLC</t>
         </is>
       </c>
-      <c r="H10" s="95" t="n"/>
-      <c r="I10" s="85" t="n"/>
-    </row>
-    <row r="11" ht="17" customFormat="1" customHeight="1" s="94">
-      <c r="A11" s="89" t="n"/>
-      <c r="B11" s="29" t="inlineStr">
+      <c r="H11" s="31" t="n"/>
+      <c r="I11" s="88" t="n"/>
+    </row>
+    <row r="12" ht="14" customFormat="1" customHeight="1" s="100">
+      <c r="A12" s="95" t="n"/>
+      <c r="B12" s="32" t="inlineStr">
         <is>
           <t>2915 N Le Compte Rd</t>
         </is>
       </c>
-      <c r="C11" s="95" t="n"/>
-      <c r="D11" s="95" t="n"/>
-      <c r="F11" s="96" t="n"/>
-      <c r="G11" s="29" t="inlineStr">
+      <c r="C12" s="101" t="n"/>
+      <c r="D12" s="88" t="n"/>
+      <c r="F12" s="102" t="n"/>
+      <c r="G12" s="32" t="inlineStr">
         <is>
           <t>2915 N Le Compte Rd</t>
         </is>
       </c>
-      <c r="H11" s="95" t="n"/>
-      <c r="I11" s="85" t="n"/>
-    </row>
-    <row r="12" ht="17" customFormat="1" customHeight="1" s="94">
-      <c r="A12" s="89" t="n"/>
-      <c r="B12" s="29" t="inlineStr">
+      <c r="H12" s="101" t="n"/>
+      <c r="I12" s="88" t="n"/>
+    </row>
+    <row r="13" ht="15.95" customFormat="1" customHeight="1" s="100">
+      <c r="A13" s="95" t="n"/>
+      <c r="B13" s="32" t="inlineStr">
         <is>
           <t>Springfield, MO 65803</t>
         </is>
       </c>
-      <c r="C12" s="95" t="n"/>
-      <c r="D12" s="95" t="n"/>
-      <c r="F12" s="96" t="n"/>
-      <c r="G12" s="29" t="inlineStr">
+      <c r="C13" s="101" t="n"/>
+      <c r="D13" s="88" t="n"/>
+      <c r="F13" s="102" t="n"/>
+      <c r="G13" s="32" t="inlineStr">
         <is>
           <t>Springfield, MO 65803</t>
         </is>
       </c>
-      <c r="H12" s="95" t="n"/>
-      <c r="I12" s="85" t="n"/>
-    </row>
-    <row r="13" ht="15.95" customFormat="1" customHeight="1" s="94">
-      <c r="A13" s="89" t="n"/>
-      <c r="B13" s="31" t="n"/>
-      <c r="C13" s="31" t="n"/>
-      <c r="D13" s="97" t="n"/>
-      <c r="F13" s="96" t="n"/>
-      <c r="G13" s="80" t="n"/>
-      <c r="H13" s="98" t="n"/>
-      <c r="I13" s="99" t="n"/>
-    </row>
-    <row r="14" ht="18.95" customFormat="1" customHeight="1" s="94">
-      <c r="A14" s="80" t="inlineStr">
+      <c r="H13" s="101" t="n"/>
+      <c r="I13" s="88" t="n"/>
+    </row>
+    <row r="14" ht="15.95" customFormat="1" customHeight="1" s="100">
+      <c r="A14" s="95" t="n"/>
+      <c r="B14" s="34" t="n"/>
+      <c r="C14" s="34" t="n"/>
+      <c r="D14" s="103" t="n"/>
+      <c r="F14" s="102" t="n"/>
+      <c r="G14" s="83" t="n"/>
+      <c r="H14" s="104" t="n"/>
+      <c r="I14" s="105" t="n"/>
+    </row>
+    <row r="15" ht="18.95" customFormat="1" customHeight="1" s="100">
+      <c r="A15" s="83" t="inlineStr">
         <is>
           <t>Port of Loading:</t>
         </is>
       </c>
-      <c r="B14" s="138" t="inlineStr">
+      <c r="B15" s="106" t="inlineStr">
         <is>
           <t>Qingdao, China</t>
         </is>
       </c>
-      <c r="F14" s="82" t="inlineStr">
+      <c r="C15" s="106" t="n"/>
+      <c r="D15" s="88" t="n"/>
+      <c r="F15" s="85" t="inlineStr">
         <is>
           <t>Actual Manufacturer Company Name</t>
         </is>
       </c>
-      <c r="G14" s="101" t="inlineStr">
+      <c r="G15" s="107" t="inlineStr">
         <is>
           <t>E MAX SPORT PTE. LTD.</t>
         </is>
       </c>
-      <c r="H14" s="102" t="n"/>
-      <c r="I14" s="85" t="n"/>
-    </row>
-    <row r="15" ht="17" customFormat="1" customHeight="1" s="94">
-      <c r="A15" s="80" t="inlineStr">
+      <c r="H15" s="108" t="n"/>
+      <c r="I15" s="88" t="n"/>
+    </row>
+    <row r="16" ht="15.95" customFormat="1" customHeight="1" s="100">
+      <c r="A16" s="83" t="inlineStr">
         <is>
           <t>Final Destination</t>
         </is>
       </c>
-      <c r="B15" s="139" t="inlineStr">
+      <c r="B16" s="109" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="F15" s="82" t="inlineStr">
+      <c r="C16" s="110" t="n"/>
+      <c r="D16" s="88" t="n"/>
+      <c r="F16" s="85" t="inlineStr">
         <is>
           <t>Actual Manufacturer Company Address</t>
         </is>
       </c>
-      <c r="G15" s="101" t="inlineStr">
+      <c r="G16" s="111" t="inlineStr">
         <is>
           <t>8 KAKI BUKIT AVENUE 4</t>
         </is>
       </c>
-      <c r="H15" s="102" t="n"/>
-      <c r="I15" s="85" t="n"/>
-    </row>
-    <row r="16" ht="29" customFormat="1" customHeight="1" s="94">
-      <c r="A16" s="89" t="n"/>
-      <c r="B16" s="97" t="n"/>
-      <c r="C16" s="97" t="n"/>
-      <c r="D16" s="97" t="n"/>
-      <c r="F16" s="96" t="n"/>
-      <c r="G16" s="106" t="inlineStr">
+      <c r="H16" s="111" t="n"/>
+      <c r="I16" s="88" t="n"/>
+    </row>
+    <row r="17" ht="24" customFormat="1" customHeight="1" s="100">
+      <c r="A17" s="95" t="n"/>
+      <c r="B17" s="103" t="n"/>
+      <c r="C17" s="103" t="n"/>
+      <c r="D17" s="103" t="n"/>
+      <c r="F17" s="102" t="n"/>
+      <c r="G17" s="112" t="inlineStr">
         <is>
           <t>#08-32,PREMIER @ KAKI BUKIT, SINGAPORE 415875</t>
         </is>
       </c>
-      <c r="H16" s="107" t="n"/>
-      <c r="I16" s="85" t="n"/>
-    </row>
-    <row r="17" ht="7" customHeight="1" s="108">
-      <c r="A17" s="109" t="n"/>
-      <c r="B17" s="110" t="n"/>
-      <c r="C17" s="110" t="n"/>
-      <c r="D17" s="110" t="n"/>
-      <c r="E17" s="110" t="n"/>
-      <c r="F17" s="110" t="n"/>
-      <c r="G17" s="110" t="n"/>
-      <c r="H17" s="110" t="n"/>
-    </row>
-    <row r="18" ht="24" customHeight="1" s="108">
-      <c r="A18" s="43" t="inlineStr">
+      <c r="H17" s="113" t="n"/>
+      <c r="I17" s="88" t="n"/>
+    </row>
+    <row r="18" ht="45" customHeight="1" s="114">
+      <c r="A18" s="115" t="n"/>
+      <c r="B18" s="116" t="n"/>
+      <c r="C18" s="116" t="n"/>
+      <c r="D18" s="116" t="n"/>
+      <c r="E18" s="116" t="n"/>
+      <c r="F18" s="116" t="n"/>
+      <c r="G18" s="116" t="n"/>
+      <c r="H18" s="116" t="n"/>
+    </row>
+    <row r="19" ht="24" customHeight="1" s="114">
+      <c r="A19" s="46" t="inlineStr">
         <is>
           <t>Country of The Origin</t>
         </is>
       </c>
-      <c r="B18" s="111" t="inlineStr">
+      <c r="B19" s="117" t="inlineStr">
         <is>
           <t>Item Number</t>
         </is>
       </c>
-      <c r="C18" s="111" t="inlineStr">
+      <c r="C19" s="117" t="inlineStr">
         <is>
           <t>UPC</t>
         </is>
       </c>
-      <c r="D18" s="45" t="inlineStr">
+      <c r="D19" s="48" t="inlineStr">
         <is>
           <t xml:space="preserve">Description </t>
         </is>
       </c>
-      <c r="E18" s="112" t="inlineStr">
+      <c r="E19" s="118" t="inlineStr">
         <is>
           <t>USD Unit Price</t>
         </is>
       </c>
-      <c r="F18" s="111" t="inlineStr">
+      <c r="F19" s="117" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="G18" s="113" t="inlineStr">
+      <c r="G19" s="119" t="inlineStr">
         <is>
           <t xml:space="preserve">USD Amount </t>
         </is>
       </c>
-      <c r="H18" s="114" t="inlineStr">
+      <c r="H19" s="120" t="inlineStr">
         <is>
           <t>EX-FACTORY DATE</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="30" customFormat="1" customHeight="1" s="73">
-      <c r="A19" s="140" t="n"/>
-      <c r="B19" s="50" t="n"/>
-      <c r="C19" s="115" t="n"/>
-      <c r="D19" s="136" t="n"/>
-      <c r="E19" s="116" t="n"/>
-      <c r="F19" s="117" t="n"/>
-      <c r="G19" s="141" t="n"/>
-      <c r="H19" s="142" t="n"/>
-    </row>
-    <row r="20" ht="30" customFormat="1" customHeight="1" s="120">
-      <c r="A20" s="140" t="n"/>
-      <c r="B20" s="50" t="n"/>
-      <c r="C20" s="115" t="n"/>
-      <c r="D20" s="136" t="n"/>
-      <c r="E20" s="116" t="n"/>
-      <c r="F20" s="117" t="n"/>
-      <c r="G20" s="141" t="n"/>
-      <c r="H20" s="142" t="n"/>
-    </row>
-    <row r="21" ht="30" customFormat="1" customHeight="1" s="120">
-      <c r="A21" s="140" t="n"/>
-      <c r="B21" s="50" t="n"/>
-      <c r="C21" s="115" t="n"/>
-      <c r="D21" s="136" t="n"/>
-      <c r="E21" s="116" t="n"/>
-      <c r="F21" s="117" t="n"/>
-      <c r="G21" s="141" t="n"/>
-      <c r="H21" s="142" t="n"/>
-    </row>
-    <row r="22" ht="30" customFormat="1" customHeight="1" s="120">
-      <c r="A22" s="140" t="n"/>
-      <c r="B22" s="50" t="n"/>
-      <c r="C22" s="115" t="n"/>
-      <c r="D22" s="136" t="n"/>
-      <c r="E22" s="116" t="n"/>
-      <c r="F22" s="117" t="n"/>
-      <c r="G22" s="141" t="n"/>
-      <c r="H22" s="142" t="n"/>
-    </row>
-    <row r="23" ht="15.95" customHeight="1" s="108">
-      <c r="A23" s="121" t="n"/>
-      <c r="B23" s="122" t="n"/>
-      <c r="C23" s="122" t="n"/>
-      <c r="D23" s="123" t="n"/>
-      <c r="E23" s="124" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sub-Total </t>
-        </is>
-      </c>
-      <c r="F23" s="61" t="n"/>
-      <c r="G23" s="62" t="n"/>
-    </row>
-    <row r="24" ht="15.95" customFormat="1" customHeight="1" s="120">
-      <c r="A24" s="125" t="n"/>
+    <row r="20" ht="17.4" customFormat="1" customHeight="1" s="76">
+      <c r="A20" s="52" t="n"/>
+      <c r="B20" s="53" t="n"/>
+      <c r="C20" s="54" t="n"/>
+      <c r="D20" s="55" t="n"/>
+      <c r="E20" s="121" t="n"/>
+      <c r="F20" s="57" t="n"/>
+      <c r="G20" s="58" t="n"/>
+      <c r="H20" s="122" t="n"/>
+    </row>
+    <row r="21" ht="17.4" customFormat="1" customHeight="1" s="123">
+      <c r="A21" s="52" t="n"/>
+      <c r="B21" s="53" t="n"/>
+      <c r="C21" s="54" t="n"/>
+      <c r="D21" s="55" t="n"/>
+      <c r="E21" s="121" t="n"/>
+      <c r="F21" s="57" t="n"/>
+      <c r="G21" s="58" t="n"/>
+      <c r="H21" s="122" t="n"/>
+    </row>
+    <row r="22" ht="17.4" customFormat="1" customHeight="1" s="123">
+      <c r="A22" s="52" t="n"/>
+      <c r="B22" s="53" t="n"/>
+      <c r="C22" s="54" t="n"/>
+      <c r="D22" s="55" t="n"/>
+      <c r="E22" s="121" t="n"/>
+      <c r="F22" s="57" t="n"/>
+      <c r="G22" s="58" t="n"/>
+      <c r="H22" s="122" t="n"/>
+    </row>
+    <row r="23" ht="17.4" customFormat="1" customHeight="1" s="123">
+      <c r="A23" s="52" t="n"/>
+      <c r="B23" s="53" t="n"/>
+      <c r="C23" s="54" t="n"/>
+      <c r="D23" s="55" t="n"/>
+      <c r="E23" s="121" t="n"/>
+      <c r="F23" s="57" t="n"/>
+      <c r="G23" s="58" t="n"/>
+      <c r="H23" s="122" t="n"/>
+    </row>
+    <row r="24" ht="15.95" customHeight="1" s="114">
+      <c r="A24" s="124" t="n"/>
       <c r="B24" s="125" t="n"/>
       <c r="C24" s="125" t="n"/>
-      <c r="D24" s="125" t="n"/>
-      <c r="F24" s="126" t="inlineStr">
+      <c r="D24" s="126" t="n"/>
+      <c r="E24" s="127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sub-Total </t>
+        </is>
+      </c>
+      <c r="F24" s="64" t="n"/>
+      <c r="G24" s="65" t="n"/>
+    </row>
+    <row r="25" ht="15.95" customFormat="1" customHeight="1" s="123">
+      <c r="A25" s="128" t="n"/>
+      <c r="B25" s="128" t="n"/>
+      <c r="C25" s="128" t="n"/>
+      <c r="D25" s="128" t="n"/>
+      <c r="F25" s="129" t="inlineStr">
         <is>
           <t>TOTAL EXCLUDING EXCISE TAX  (USD)</t>
         </is>
       </c>
-      <c r="G24" s="65" t="n"/>
-      <c r="H24" s="127" t="n"/>
-    </row>
-    <row r="25" ht="15.95" customFormat="1" customHeight="1" s="120">
-      <c r="H25" s="127" t="n"/>
-    </row>
-    <row r="26" ht="15.95" customFormat="1" customHeight="1" s="120">
-      <c r="A26" s="128" t="n"/>
-      <c r="E26" s="129" t="inlineStr">
+      <c r="G25" s="68" t="n"/>
+      <c r="H25" s="130" t="n"/>
+    </row>
+    <row r="26" ht="15.95" customFormat="1" customHeight="1" s="123">
+      <c r="H26" s="130" t="n"/>
+    </row>
+    <row r="27" ht="15.95" customFormat="1" customHeight="1" s="123">
+      <c r="A27" s="131" t="n"/>
+      <c r="E27" s="132" t="inlineStr">
         <is>
           <t>Signature:</t>
         </is>
       </c>
-      <c r="F26" s="130" t="n"/>
-      <c r="G26" s="130" t="n"/>
-      <c r="H26" s="85" t="n"/>
-    </row>
-    <row r="27" ht="15.95" customFormat="1" customHeight="1" s="120">
-      <c r="A27" s="128" t="n"/>
-      <c r="E27" s="131" t="inlineStr">
+      <c r="F27" s="133" t="n"/>
+      <c r="G27" s="133" t="n"/>
+      <c r="H27" s="88" t="n"/>
+    </row>
+    <row r="28" ht="15.95" customFormat="1" customHeight="1" s="123">
+      <c r="A28" s="131" t="n"/>
+      <c r="E28" s="134" t="inlineStr">
         <is>
           <t>Date:</t>
         </is>
       </c>
-      <c r="F27" s="132" t="n"/>
-      <c r="G27" s="133" t="n"/>
-      <c r="H27" s="85" t="n"/>
-    </row>
-    <row r="28" customFormat="1" s="120">
-      <c r="H28" s="127" t="n"/>
+      <c r="F28" s="135" t="n"/>
+      <c r="G28" s="136" t="n"/>
+      <c r="H28" s="88" t="n"/>
+    </row>
+    <row r="29" customFormat="1" s="123">
+      <c r="H29" s="130" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="B11:D11"/>
+  <mergeCells count="9">
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="A4:H4"/>
     <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="G6:H6"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="G15:H15"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="G16:H16"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="B12:C12"/>
   </mergeCells>
-  <conditionalFormatting sqref="B19">
+  <conditionalFormatting sqref="B20">
     <cfRule type="duplicateValues" priority="3" dxfId="0"/>
     <cfRule type="duplicateValues" priority="4" dxfId="0"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B20:B22">
+  <conditionalFormatting sqref="B21:B23">
     <cfRule type="duplicateValues" priority="1" dxfId="0"/>
     <cfRule type="duplicateValues" priority="2" dxfId="0"/>
   </conditionalFormatting>
   <pageMargins left="0.196850393700787" right="0.236220472440945" top="0.275590551181102" bottom="0.31496062992126" header="0.236220472440945" footer="0.196850393700787"/>
-  <pageSetup orientation="portrait" paperSize="1" scale="80" verticalDpi="203"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="76" verticalDpi="203"/>
 </worksheet>
 </file>
</xml_diff>